<commit_message>
did work on the PPO and A2C models
</commit_message>
<xml_diff>
--- a/Time Sheet.xlsx
+++ b/Time Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninja\School\Atari-Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C34219C-1F47-4BAC-92B7-A777F4F1D24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A17D40-66FC-422F-BF9B-B20CF9CF6B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F056FDBC-FD1C-4AAD-B5EB-AB9B4822F501}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
   <si>
     <t>HOURS</t>
   </si>
@@ -117,6 +117,12 @@
   </si>
   <si>
     <t>fixed loader.</t>
+  </si>
+  <si>
+    <t>learned a2c and ppo</t>
+  </si>
+  <si>
+    <t>worked more on PPO model</t>
   </si>
 </sst>
 </file>
@@ -155,10 +161,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA24217B-B1AF-4ADA-826D-205E5762FA65}">
-  <dimension ref="A2:P21"/>
+  <dimension ref="A2:P23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -547,7 +554,7 @@
       </c>
       <c r="M4" s="1">
         <f>SUM(C:C)</f>
-        <v>1.5902777777777777</v>
+        <v>1.6944444444444442</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -565,7 +572,7 @@
       </c>
       <c r="M5" s="1">
         <f>M3-M4</f>
-        <v>2.1597222222222223</v>
+        <v>2.0555555555555558</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -742,6 +749,28 @@
       </c>
       <c r="E21" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>46088</v>
+      </c>
+      <c r="C22" s="1">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>46089</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more statistocsamong a few other few things
</commit_message>
<xml_diff>
--- a/Time Sheet.xlsx
+++ b/Time Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninja\School\Atari-Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A17D40-66FC-422F-BF9B-B20CF9CF6B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0552DDFF-D74C-4203-80FE-8E5B8A15BF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F056FDBC-FD1C-4AAD-B5EB-AB9B4822F501}"/>
   </bookViews>
@@ -554,7 +554,7 @@
       </c>
       <c r="M4" s="1">
         <f>SUM(C:C)</f>
-        <v>1.6944444444444442</v>
+        <v>1.7569444444444442</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -572,7 +572,7 @@
       </c>
       <c r="M5" s="1">
         <f>M3-M4</f>
-        <v>2.0555555555555558</v>
+        <v>1.9930555555555558</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -767,7 +767,7 @@
         <v>46089</v>
       </c>
       <c r="C23" s="1">
-        <v>2.0833333333333332E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="E23" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
updated PPO code. still have work to do
</commit_message>
<xml_diff>
--- a/Time Sheet.xlsx
+++ b/Time Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninja\School\Atari-Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0552DDFF-D74C-4203-80FE-8E5B8A15BF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B581C32A-0BC9-4105-829A-A82D9F56D181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F056FDBC-FD1C-4AAD-B5EB-AB9B4822F501}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="20136" windowHeight="11232" xr2:uid="{F056FDBC-FD1C-4AAD-B5EB-AB9B4822F501}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>HOURS</t>
   </si>
@@ -123,6 +123,21 @@
   </si>
   <si>
     <t>worked more on PPO model</t>
+  </si>
+  <si>
+    <t>bug fixing and few minor changes</t>
+  </si>
+  <si>
+    <t>working on chart code and other statistics</t>
+  </si>
+  <si>
+    <t>ran some tests and to verify changes made didn’t crash the code</t>
+  </si>
+  <si>
+    <t>fixed my statistics and made some other changes.</t>
+  </si>
+  <si>
+    <t>added stats to PPO</t>
   </si>
 </sst>
 </file>
@@ -161,11 +176,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,12 +516,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA24217B-B1AF-4ADA-826D-205E5762FA65}">
-  <dimension ref="A2:P23"/>
+  <dimension ref="A2:P28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -535,6 +552,9 @@
       <c r="M3" s="1">
         <v>3.75</v>
       </c>
+      <c r="N3" s="4">
+        <v>6.25</v>
+      </c>
       <c r="P3" t="s">
         <v>24</v>
       </c>
@@ -554,7 +574,11 @@
       </c>
       <c r="M4" s="1">
         <f>SUM(C:C)</f>
-        <v>1.7569444444444442</v>
+        <v>2.2569444444444442</v>
+      </c>
+      <c r="N4" s="1">
+        <f>SUM(C:C)</f>
+        <v>2.2569444444444442</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -572,7 +596,11 @@
       </c>
       <c r="M5" s="1">
         <f>M3-M4</f>
-        <v>1.9930555555555558</v>
+        <v>1.4930555555555558</v>
+      </c>
+      <c r="N5" s="1">
+        <f>N3-N4</f>
+        <v>3.9930555555555558</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -771,6 +799,61 @@
       </c>
       <c r="E23" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>46092</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>46093</v>
+      </c>
+      <c r="C25" s="1">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>46094</v>
+      </c>
+      <c r="C26" s="1">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>46095</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="E27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>46100</v>
+      </c>
+      <c r="C28" s="1">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>